<commit_message>
Add HKS testlop 2026-04-30 results
</commit_message>
<xml_diff>
--- a/Testløp/data/2026_HKS_Testlop_Resultater_Pamelding_Hjelpere.xlsx
+++ b/Testløp/data/2026_HKS_Testlop_Resultater_Pamelding_Hjelpere.xlsx
@@ -8,6 +8,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HKS 2026-04-23 Løp #2" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HKS 2026-04-25 Løp #3" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HKS 2026-04-28 Løp #4" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HKS 2026-04-30 Løp #5" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'HKS 2026-04-18 Løp #1'!$C$18:$D$23</definedName>
@@ -651,7 +652,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.5" customWidth="1" style="56" min="1" max="1"/>
@@ -704,18 +705,25 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n"/>
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>HKS 2026-04-30 Løp #5</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Antall resulater:</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>tba</t>
         </is>
@@ -2018,7 +2026,7 @@
       <c r="D9" s="21" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="0" t="inlineStr">
         <is>
           <t>Amalie Tolcsiner</t>
         </is>
@@ -2069,7 +2077,6 @@
       <c r="C15" s="26" t="n"/>
       <c r="D15" s="27" t="n"/>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="48" t="inlineStr">
         <is>
@@ -2176,4 +2183,300 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape" paperSize="9" scale="120" pageOrder="overThenDown" cellComments="atEnd"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:D33"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="30.13" customWidth="1" style="56" min="1" max="1"/>
+    <col width="6.75" customWidth="1" style="56" min="2" max="2"/>
+    <col width="22.13" customWidth="1" style="56" min="3" max="3"/>
+    <col width="6.5" customWidth="1" style="56" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="n"/>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Kommentar</t>
+        </is>
+      </c>
+      <c r="C1" s="57" t="n"/>
+      <c r="D1" s="13" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>Gustav</t>
+        </is>
+      </c>
+      <c r="B2" s="46" t="inlineStr">
+        <is>
+          <t>Hjelper</t>
+        </is>
+      </c>
+      <c r="D2" s="58" t="n"/>
+    </row>
+    <row r="3">
+      <c r="B3" s="46" t="inlineStr">
+        <is>
+          <t>Hjelper</t>
+        </is>
+      </c>
+      <c r="D3" s="58" t="n"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="46" t="inlineStr">
+        <is>
+          <t>Hjelper</t>
+        </is>
+      </c>
+      <c r="D4" s="58" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>HKS #5 Torsdagsstestl?p 30.04.2026 - 
+600m og 1200m</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Fritt skovalg</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="59" t="inlineStr">
+        <is>
+          <t>Skriv inn ditt navn</t>
+        </is>
+      </c>
+      <c r="D7" s="58" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>600m - Kvinner kl10:15-20</t>
+        </is>
+      </c>
+      <c r="C8" s="63" t="inlineStr">
+        <is>
+          <t>1200m - Kvinner kl10:15-20</t>
+        </is>
+      </c>
+      <c r="D8" s="58" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>Navn</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="n"/>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>Navn</t>
+        </is>
+      </c>
+      <c r="D9" s="34" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="54" t="inlineStr">
+        <is>
+          <t>Gioia Chiesurin</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>1:49,3</t>
+        </is>
+      </c>
+      <c r="C10" s="38" t="inlineStr">
+        <is>
+          <t>Ine Bakken</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>3:35,8</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>Noa Antonissen</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>1:55,7</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>Mathilde Knutsen</t>
+        </is>
+      </c>
+      <c r="D11" s="27" t="inlineStr">
+        <is>
+          <t>3:40,1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>Celeste van Essen</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>1:59,6</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="n"/>
+      <c r="D12" s="27" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>Michelle Geertse</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>2:05,4</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="n"/>
+      <c r="D13" s="27" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="26" t="n"/>
+      <c r="B14" s="26" t="n"/>
+      <c r="C14" s="26" t="n"/>
+      <c r="D14" s="27" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="n"/>
+      <c r="B15" s="26" t="n"/>
+      <c r="C15" s="26" t="n"/>
+      <c r="D15" s="27" t="n"/>
+    </row>
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="48" t="inlineStr">
+        <is>
+          <t>600m - Menn kl10:15-20</t>
+        </is>
+      </c>
+      <c r="C17" s="60" t="inlineStr">
+        <is>
+          <t>1200m - Menn kl10:15-20</t>
+        </is>
+      </c>
+      <c r="D17" s="58" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>Navn</t>
+        </is>
+      </c>
+      <c r="B18" s="21" t="n"/>
+      <c r="C18" s="21" t="inlineStr">
+        <is>
+          <t>Navn</t>
+        </is>
+      </c>
+      <c r="D18" s="34" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>Simen Hagerup Kjeldsen</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>1:53,5</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>Gunnar Berthelsen</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>4:32,3</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="26" t="n"/>
+      <c r="B20" s="26" t="n"/>
+      <c r="C20" s="26" t="n"/>
+      <c r="D20" s="27" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="26" t="n"/>
+      <c r="B21" s="26" t="n"/>
+      <c r="C21" s="26" t="n"/>
+      <c r="D21" s="27" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="54" t="n"/>
+      <c r="B22" s="26" t="n"/>
+      <c r="C22" s="26" t="n"/>
+      <c r="D22" s="27" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="26" t="n"/>
+      <c r="B23" s="26" t="n"/>
+      <c r="C23" s="26" t="n"/>
+      <c r="D23" s="27" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="54" t="n"/>
+      <c r="B24" s="54" t="n"/>
+      <c r="C24" s="54" t="n"/>
+    </row>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="B2:D2"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1" gridLines="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" pageOrder="overThenDown" cellComments="atEnd"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add HKS testlop 2026-04-30 PM results
</commit_message>
<xml_diff>
--- a/Testløp/data/2026_HKS_Testlop_Resultater_Pamelding_Hjelpere.xlsx
+++ b/Testløp/data/2026_HKS_Testlop_Resultater_Pamelding_Hjelpere.xlsx
@@ -9,6 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HKS 2026-04-25 Løp #3" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HKS 2026-04-28 Løp #4" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HKS 2026-04-30 Løp #5" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HKS 2026-04-30 Løp #6 p.m." sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'HKS 2026-04-18 Løp #1'!$C$18:$D$23</definedName>
@@ -652,7 +653,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.5" customWidth="1" style="56" min="1" max="1"/>
@@ -665,7 +666,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -712,18 +712,25 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>HKS 2026-04-30 Løp #6 p.m.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Antall resulater:</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>tba</t>
         </is>
@@ -2191,7 +2198,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="30.13" customWidth="1" style="56" min="1" max="1"/>
@@ -2373,7 +2380,6 @@
       <c r="C15" s="26" t="n"/>
       <c r="D15" s="27" t="n"/>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="48" t="inlineStr">
         <is>
@@ -2452,15 +2458,352 @@
       <c r="B24" s="54" t="n"/>
       <c r="C24" s="54" t="n"/>
     </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="B2:D2"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1" gridLines="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" pageOrder="overThenDown" cellComments="atEnd"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="30.13" customWidth="1" style="56" min="1" max="1"/>
+    <col width="6.75" customWidth="1" style="56" min="2" max="2"/>
+    <col width="22.13" customWidth="1" style="56" min="3" max="3"/>
+    <col width="6.5" customWidth="1" style="56" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="n"/>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Kommentar</t>
+        </is>
+      </c>
+      <c r="C1" s="57" t="n"/>
+      <c r="D1" s="13" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>Gustav</t>
+        </is>
+      </c>
+      <c r="B2" s="46" t="inlineStr">
+        <is>
+          <t>Hjelper</t>
+        </is>
+      </c>
+      <c r="D2" s="58" t="n"/>
+    </row>
+    <row r="3">
+      <c r="B3" s="46" t="inlineStr">
+        <is>
+          <t>Hjelper</t>
+        </is>
+      </c>
+      <c r="D3" s="58" t="n"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="46" t="inlineStr">
+        <is>
+          <t>Hjelper</t>
+        </is>
+      </c>
+      <c r="D4" s="58" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>HKS #6 Torsdagstestl?p 30.04.2026 p.m. - 
+600m og 1200m</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Fritt skovalg</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="59" t="inlineStr">
+        <is>
+          <t>Skriv inn ditt navn</t>
+        </is>
+      </c>
+      <c r="D7" s="58" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>600m - Kvinner</t>
+        </is>
+      </c>
+      <c r="C8" s="63" t="inlineStr">
+        <is>
+          <t>1200m - Kvinner</t>
+        </is>
+      </c>
+      <c r="D8" s="58" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>Navn</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="n"/>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>Navn</t>
+        </is>
+      </c>
+      <c r="D9" s="34" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="54" t="inlineStr">
+        <is>
+          <t>Telma Eckhoff Dagestad</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>1:43,2</t>
+        </is>
+      </c>
+      <c r="C10" s="38" t="inlineStr">
+        <is>
+          <t>Frida Konow</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>3:35,9</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>Ingrid Rustad Røflo</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>1:44,9</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="n"/>
+      <c r="D11" s="27" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>Mai Watson</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>1:45,9</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="n"/>
+      <c r="D12" s="27" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="26" t="n"/>
+      <c r="B13" s="26" t="n"/>
+      <c r="C13" s="26" t="n"/>
+      <c r="D13" s="27" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="26" t="n"/>
+      <c r="B14" s="26" t="n"/>
+      <c r="C14" s="26" t="n"/>
+      <c r="D14" s="27" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="n"/>
+      <c r="B15" s="26" t="n"/>
+      <c r="C15" s="26" t="n"/>
+      <c r="D15" s="27" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="48" t="inlineStr">
+        <is>
+          <t>600m - Menn</t>
+        </is>
+      </c>
+      <c r="C17" s="60" t="inlineStr">
+        <is>
+          <t>1200m - Menn</t>
+        </is>
+      </c>
+      <c r="D17" s="58" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>Navn</t>
+        </is>
+      </c>
+      <c r="B18" s="21" t="n"/>
+      <c r="C18" s="21" t="inlineStr">
+        <is>
+          <t>Navn</t>
+        </is>
+      </c>
+      <c r="D18" s="34" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>Riley McGown</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>1:24,9</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>Haakon Engelsen Berg</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>3:14,2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>Emil Skogheim</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>1:34,7</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>Erlend Sørtveit</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="inlineStr">
+        <is>
+          <t>3:15,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>Jørgen Engøy</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>1:37,5</t>
+        </is>
+      </c>
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>Kristian Stenerud</t>
+        </is>
+      </c>
+      <c r="D21" s="27" t="inlineStr">
+        <is>
+          <t>3:32,6</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="54" t="inlineStr">
+        <is>
+          <t>Simen Modin Engesæth</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>1:39,1</t>
+        </is>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>Erlend Aune</t>
+        </is>
+      </c>
+      <c r="D22" s="27" t="inlineStr">
+        <is>
+          <t>3:50,1</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>Fredrik Camilo Halsbog</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>1:40,7</t>
+        </is>
+      </c>
+      <c r="C23" s="26" t="n"/>
+      <c r="D23" s="27" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="54" t="inlineStr">
+        <is>
+          <t>Adam Olsen</t>
+        </is>
+      </c>
+      <c r="B24" s="54" t="inlineStr">
+        <is>
+          <t>1:42,0</t>
+        </is>
+      </c>
+      <c r="C24" s="54" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>Shervin Fashkhami</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>1:46,3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="A5:D5"/>

</xml_diff>

<commit_message>
Add HKS testlop 2026-05-02 results
</commit_message>
<xml_diff>
--- a/Testløp/data/2026_HKS_Testlop_Resultater_Pamelding_Hjelpere.xlsx
+++ b/Testløp/data/2026_HKS_Testlop_Resultater_Pamelding_Hjelpere.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HKS 2026-04-28 Løp #4" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HKS 2026-04-30 Løp #5" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HKS 2026-04-30 Løp #6 p.m." sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HKS 2026-05-02 Løp #7" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'HKS 2026-04-18 Løp #1'!$C$18:$D$23</definedName>
@@ -653,7 +654,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.5" customWidth="1" style="56" min="1" max="1"/>
@@ -666,6 +667,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -719,18 +721,25 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n"/>
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>HKS 2026-05-02 Løp #7</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Antall resulater:</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>tba</t>
         </is>
@@ -2822,4 +2831,353 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" pageOrder="overThenDown" cellComments="atEnd"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:D26"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="30.13" customWidth="1" style="56" min="1" max="1"/>
+    <col width="6.75" customWidth="1" style="56" min="2" max="2"/>
+    <col width="22.13" customWidth="1" style="56" min="3" max="3"/>
+    <col width="6.5" customWidth="1" style="56" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="n"/>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Kommentar</t>
+        </is>
+      </c>
+      <c r="C1" s="57" t="n"/>
+      <c r="D1" s="13" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>Gustav</t>
+        </is>
+      </c>
+      <c r="B2" s="46" t="inlineStr">
+        <is>
+          <t>Hjelper</t>
+        </is>
+      </c>
+      <c r="D2" s="58" t="n"/>
+    </row>
+    <row r="3">
+      <c r="B3" s="46" t="inlineStr">
+        <is>
+          <t>Hjelper</t>
+        </is>
+      </c>
+      <c r="D3" s="58" t="n"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="46" t="inlineStr">
+        <is>
+          <t>Hjelper</t>
+        </is>
+      </c>
+      <c r="D4" s="58" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>HKS #7 Lørdagsstestløp 02.05.2026 - 
+600m og 1200m</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Fritt skovalg</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="59" t="inlineStr">
+        <is>
+          <t>Skriv inn ditt navn</t>
+        </is>
+      </c>
+      <c r="D7" s="58" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>600m - Kvinner kl10:10</t>
+        </is>
+      </c>
+      <c r="C8" s="63" t="inlineStr">
+        <is>
+          <t>1200m - Kvinner kl10:15</t>
+        </is>
+      </c>
+      <c r="D8" s="58" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>Navn</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="n"/>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>Navn</t>
+        </is>
+      </c>
+      <c r="D9" s="34" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="54" t="inlineStr">
+        <is>
+          <t>Telma Eckhoff Dagestad</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>1:30,1</t>
+        </is>
+      </c>
+      <c r="C10" s="38" t="inlineStr">
+        <is>
+          <t>Sofie Amundsgård</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>3:52,4</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>Vilde Antonsen</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>1:36,6</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>Live Maria Grønvold</t>
+        </is>
+      </c>
+      <c r="D11" s="27" t="inlineStr">
+        <is>
+          <t>4:19,6</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>Mai Watson</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>1:44,6</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="n"/>
+      <c r="D12" s="27" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>Synne Amundsgård</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>1:48,1</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="n"/>
+      <c r="D13" s="27" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>Victoria Rochelois</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>2:16,6</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="n"/>
+      <c r="D14" s="27" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="n"/>
+      <c r="B15" s="26" t="n"/>
+      <c r="C15" s="26" t="n"/>
+      <c r="D15" s="27" t="n"/>
+    </row>
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="48" t="inlineStr">
+        <is>
+          <t>600m - Menn kl10:10</t>
+        </is>
+      </c>
+      <c r="C17" s="60" t="inlineStr">
+        <is>
+          <t>1200m - Menn kl10:15</t>
+        </is>
+      </c>
+      <c r="D17" s="58" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>Navn</t>
+        </is>
+      </c>
+      <c r="B18" s="21" t="n"/>
+      <c r="C18" s="21" t="inlineStr">
+        <is>
+          <t>Navn</t>
+        </is>
+      </c>
+      <c r="D18" s="34" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>Henrik Hansen</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>1:32,30</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>Trond Einar Pedersli</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>3:12,2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>Børge Bårdsen</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>1:47,2</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>Mathias Moen</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="inlineStr">
+        <is>
+          <t>3:15,9</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="26" t="n"/>
+      <c r="B21" s="26" t="n"/>
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>Anton Heldal</t>
+        </is>
+      </c>
+      <c r="D21" s="27" t="inlineStr">
+        <is>
+          <t>3:18,2</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="54" t="n"/>
+      <c r="B22" s="26" t="n"/>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>Eivind Bækkedal</t>
+        </is>
+      </c>
+      <c r="D22" s="27" t="inlineStr">
+        <is>
+          <t>3:31,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="26" t="n"/>
+      <c r="B23" s="26" t="n"/>
+      <c r="C23" s="26" t="inlineStr">
+        <is>
+          <t>Erik Bucher Johannessen</t>
+        </is>
+      </c>
+      <c r="D23" s="27" t="inlineStr">
+        <is>
+          <t>3:38,4</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="54" t="n"/>
+      <c r="B24" s="54" t="n"/>
+      <c r="C24" s="54" t="inlineStr">
+        <is>
+          <t>Sondre Kongsgård</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>4:00,9</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n"/>
+      <c r="B25" s="0" t="n"/>
+    </row>
+    <row r="26"/>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="B2:D2"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1" gridLines="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" pageOrder="overThenDown" cellComments="atEnd"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix Telma HKS 7 time
</commit_message>
<xml_diff>
--- a/Testløp/data/2026_HKS_Testlop_Resultater_Pamelding_Hjelpere.xlsx
+++ b/Testløp/data/2026_HKS_Testlop_Resultater_Pamelding_Hjelpere.xlsx
@@ -667,7 +667,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -2839,7 +2838,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="30.13" customWidth="1" style="56" min="1" max="1"/>
@@ -2945,7 +2944,7 @@
       </c>
       <c r="B10" s="26" t="inlineStr">
         <is>
-          <t>1:30,1</t>
+          <t>1:40,1</t>
         </is>
       </c>
       <c r="C10" s="38" t="inlineStr">
@@ -3151,7 +3150,7 @@
           <t>Sondre Kongsgård</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>4:00,9</t>
         </is>
@@ -3161,7 +3160,6 @@
       <c r="A25" s="0" t="n"/>
       <c r="B25" s="0" t="n"/>
     </row>
-    <row r="26"/>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="A5:D5"/>

</xml_diff>